<commit_message>
🚀 Updated framework with latest changes: parallel browser support, Allure fixes, report automation
</commit_message>
<xml_diff>
--- a/OrderIDs.xlsx
+++ b/OrderIDs.xlsx
@@ -17,13 +17,13 @@
     <t>Order ID</t>
   </si>
   <si>
-    <t>QIX-1201</t>
+    <t>QIX-1868</t>
   </si>
   <si>
-    <t>QIX-1202</t>
+    <t>QIX-1869</t>
   </si>
   <si>
-    <t>QIX-1203</t>
+    <t>QIX-1870</t>
   </si>
 </sst>
 </file>

</xml_diff>